<commit_message>
Update 김청축_2026_출석부.xlsx via Dashboard
</commit_message>
<xml_diff>
--- a/김청축_2026_출석부.xlsx
+++ b/김청축_2026_출석부.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Han\codes\kcc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2B2B9F-0C5A-48DA-8C47-99FB3E118D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B99574-741D-41AE-9FEE-F076AF182266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="606" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="606" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="종합Sheet" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1331" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1328" uniqueCount="370">
   <si>
     <t>C/S DF (0.2)</t>
   </si>
@@ -2167,10 +2167,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2179,20 +2179,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="H2" s="18">
         <f>SUM(J2:AR2)/COUNTA(J2:BB2)</f>
-        <v>3.0666666666666669</v>
+        <v>3.0444444444444443</v>
       </c>
       <c r="I2" s="18" t="s">
         <v>83</v>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="P2" s="1">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Q2" s="1">
         <f t="shared" si="0"/>
@@ -3447,7 +3447,7 @@
       </c>
       <c r="G5" s="2">
         <f>RANK(H5,$H$4:$H$122,0)</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H5" s="6">
         <f>I5+개인기록Sheet!C5</f>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="G11" s="2">
         <f t="shared" si="4"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H11" s="6">
         <f>I11+개인기록Sheet!C11</f>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="G16" s="2">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H16" s="6">
         <f>I16+개인기록Sheet!C16</f>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="G17" s="2">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H17" s="6">
         <f>I17+개인기록Sheet!C17</f>
@@ -5018,7 +5018,7 @@
       </c>
       <c r="G20" s="2">
         <f t="shared" si="4"/>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H20" s="6">
         <f>I20+개인기록Sheet!C20</f>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="G25" s="2">
         <f t="shared" si="4"/>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H25" s="6">
         <f>I25+개인기록Sheet!C25</f>
@@ -5753,7 +5753,7 @@
       </c>
       <c r="G27" s="2">
         <f t="shared" si="4"/>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H27" s="6">
         <f>I27+개인기록Sheet!C27</f>
@@ -6163,7 +6163,7 @@
       </c>
       <c r="G31" s="2">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H31" s="6">
         <f>I31+개인기록Sheet!C31</f>
@@ -6270,7 +6270,7 @@
       </c>
       <c r="G32" s="2">
         <f t="shared" si="4"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H32" s="6">
         <f>I32+개인기록Sheet!C32</f>
@@ -7021,7 +7021,7 @@
       </c>
       <c r="G39" s="2">
         <f t="shared" si="4"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H39" s="6">
         <f>I39+개인기록Sheet!C39</f>
@@ -7130,7 +7130,7 @@
       </c>
       <c r="G40" s="2">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H40" s="6">
         <f>I40+개인기록Sheet!C40</f>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="G47" s="2">
         <f t="shared" si="4"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H47" s="6">
         <f>I47+개인기록Sheet!C47</f>
@@ -8269,7 +8269,7 @@
       </c>
       <c r="G51" s="2">
         <f t="shared" si="4"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H51" s="6">
         <f>I51+개인기록Sheet!C51</f>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="G56" s="2">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H56" s="6">
         <f>I56+개인기록Sheet!C56</f>
@@ -9723,7 +9723,7 @@
       </c>
       <c r="G65" s="2">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H65" s="6">
         <f>I65+개인기록Sheet!C65</f>
@@ -9830,7 +9830,7 @@
       </c>
       <c r="G66" s="2">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H66" s="6">
         <f>I66+개인기록Sheet!C66</f>
@@ -9937,7 +9937,7 @@
       </c>
       <c r="G67" s="2">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H67" s="6">
         <f>I67+개인기록Sheet!C67</f>
@@ -10145,7 +10145,7 @@
       </c>
       <c r="G69" s="2">
         <f t="shared" si="4"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H69" s="6">
         <f>I69+개인기록Sheet!C69</f>
@@ -10355,7 +10355,7 @@
       </c>
       <c r="G71" s="2">
         <f t="shared" ref="G71:G114" si="6">RANK(H71,$H$4:$H$122,0)</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H71" s="6">
         <f>I71+개인기록Sheet!C71</f>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="G74" s="2">
         <f t="shared" si="6"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H74" s="6">
         <f>I74+개인기록Sheet!C74</f>
@@ -10769,7 +10769,7 @@
       </c>
       <c r="G75" s="2">
         <f t="shared" si="6"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H75" s="6">
         <f>I75+개인기록Sheet!C75</f>
@@ -12324,7 +12324,7 @@
       </c>
       <c r="G90" s="2">
         <f t="shared" si="6"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H90" s="6">
         <f>I90+개인기록Sheet!C90</f>
@@ -12637,7 +12637,7 @@
       </c>
       <c r="G93" s="2">
         <f t="shared" si="6"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H93" s="6">
         <f>I93+개인기록Sheet!C93</f>
@@ -13394,7 +13394,7 @@
       </c>
       <c r="G100" s="2">
         <f t="shared" si="6"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H100" s="6">
         <f>I100+개인기록Sheet!C100</f>
@@ -13501,15 +13501,15 @@
       </c>
       <c r="G101" s="2">
         <f t="shared" si="6"/>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H101" s="6">
         <f>I101+개인기록Sheet!C101</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I101" s="6">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J101" s="2" t="s">
         <v>355</v>
@@ -13523,9 +13523,7 @@
       <c r="O101" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="P101" s="2" t="s">
-        <v>205</v>
-      </c>
+      <c r="P101" s="2"/>
       <c r="Q101" s="2"/>
       <c r="R101" s="2"/>
       <c r="S101" s="2"/>
@@ -13612,7 +13610,7 @@
       </c>
       <c r="G102" s="2">
         <f t="shared" si="6"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H102" s="6">
         <f>I102+개인기록Sheet!C102</f>
@@ -13719,11 +13717,11 @@
       </c>
       <c r="G103" s="2">
         <f t="shared" si="6"/>
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H103" s="6">
         <f>I103+개인기록Sheet!C103</f>
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="I103" s="6">
         <f t="shared" si="7"/>
@@ -13929,7 +13927,7 @@
       </c>
       <c r="G105" s="2">
         <f t="shared" si="6"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H105" s="6">
         <f>I105+개인기록Sheet!C105</f>
@@ -14036,7 +14034,7 @@
       </c>
       <c r="G106" s="2">
         <f t="shared" si="6"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H106" s="6">
         <f>I106+개인기록Sheet!C106</f>
@@ -15586,12 +15584,8 @@
       <c r="N20" s="20" t="s">
         <v>309</v>
       </c>
-      <c r="O20" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="P20" s="20" t="s">
-        <v>230</v>
-      </c>
+      <c r="O20" s="20"/>
+      <c r="P20" s="20"/>
       <c r="Q20" s="9" t="s">
         <v>137</v>
       </c>
@@ -15657,6 +15651,29 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="Q2:V2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="I13:L13"/>
+    <mergeCell ref="M13:P13"/>
+    <mergeCell ref="Q13:V13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="D20:D21"/>
@@ -15666,29 +15683,6 @@
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E13:H13"/>
-    <mergeCell ref="I13:L13"/>
-    <mergeCell ref="M13:P13"/>
-    <mergeCell ref="Q13:V13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="Q2:V2"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.74805557727813721" right="0.74805557727813721" top="0.98430556058883667" bottom="0.98430556058883667" header="0.51138889789581299" footer="0.51138889789581299"/>
@@ -19931,7 +19925,7 @@
         <v>정재명</v>
       </c>
       <c r="C100" s="2">
-        <f t="shared" ref="C100:C131" si="11">((D100+E100+G100+H100)*0.2)+(F100*0.3)</f>
+        <f t="shared" ref="C100:C114" si="11">((D100+E100+G100+H100)*0.2)+(F100*0.3)</f>
         <v>0</v>
       </c>
       <c r="D100" s="14">
@@ -19955,7 +19949,7 @@
         <v>0</v>
       </c>
       <c r="I100" s="14">
-        <f t="shared" ref="I100:I131" si="12">SUM(D100:H100)</f>
+        <f t="shared" ref="I100:I114" si="12">SUM(D100:H100)</f>
         <v>0</v>
       </c>
       <c r="J100" s="15"/>
@@ -20049,7 +20043,7 @@
       </c>
       <c r="C103" s="2">
         <f t="shared" si="11"/>
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D103" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B103)</f>
@@ -20061,7 +20055,7 @@
       </c>
       <c r="F103" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B103)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G103" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B103)</f>
@@ -20073,7 +20067,7 @@
       </c>
       <c r="I103" s="14">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J103" s="15"/>
     </row>
@@ -22084,10 +22078,10 @@
       <c r="G2" s="48" t="s">
         <v>334</v>
       </c>
-      <c r="I2" s="99" t="s">
+      <c r="I2" s="94" t="s">
         <v>249</v>
       </c>
-      <c r="J2" s="99"/>
+      <c r="J2" s="94"/>
       <c r="K2" s="66" t="s">
         <v>277</v>
       </c>
@@ -22112,7 +22106,7 @@
       </c>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B3" s="100" t="s">
+      <c r="B3" s="93" t="s">
         <v>340</v>
       </c>
       <c r="C3" s="73">
@@ -22328,7 +22322,7 @@
         <f>VLOOKUP(F7,종합Sheet!$B$3:$I$114,7,0)</f>
         <v>5</v>
       </c>
-      <c r="I7" s="97"/>
+      <c r="I7" s="98"/>
       <c r="J7" s="67">
         <v>5</v>
       </c>
@@ -22414,10 +22408,10 @@
         <f>VLOOKUP(F9,종합Sheet!$B$3:$I$114,7,0)</f>
         <v>1</v>
       </c>
-      <c r="I9" s="99" t="s">
+      <c r="I9" s="94" t="s">
         <v>249</v>
       </c>
-      <c r="J9" s="99"/>
+      <c r="J9" s="94"/>
       <c r="K9" s="66" t="s">
         <v>277</v>
       </c>
@@ -22538,7 +22532,7 @@
       </c>
       <c r="S11" s="72">
         <f>VLOOKUP(R11,종합Sheet!$B$3:$I$114,7,0)</f>
-        <v>2.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.25">
@@ -22570,7 +22564,7 @@
       <c r="L12" s="66">
         <v>8</v>
       </c>
-      <c r="N12" s="98"/>
+      <c r="N12" s="101"/>
       <c r="O12" s="49">
         <v>10</v>
       </c>
@@ -22644,7 +22638,7 @@
         <f>VLOOKUP(F14,종합Sheet!$B$3:$I$114,7,0)</f>
         <v>5</v>
       </c>
-      <c r="I14" s="97"/>
+      <c r="I14" s="98"/>
       <c r="J14" s="67">
         <v>5</v>
       </c>
@@ -22707,10 +22701,10 @@
         <v>3</v>
       </c>
       <c r="H16" s="38"/>
-      <c r="I16" s="99" t="s">
+      <c r="I16" s="94" t="s">
         <v>249</v>
       </c>
-      <c r="J16" s="99"/>
+      <c r="J16" s="94"/>
       <c r="K16" s="66" t="s">
         <v>277</v>
       </c>
@@ -22733,7 +22727,7 @@
       </c>
       <c r="G17" s="64">
         <f>VLOOKUP(F17,종합Sheet!$B$3:$I$114,7,0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H17" s="38"/>
       <c r="I17" s="95" t="s">
@@ -22771,10 +22765,10 @@
       <c r="U18"/>
     </row>
     <row r="19" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B19" s="99" t="s">
+      <c r="B19" s="94" t="s">
         <v>249</v>
       </c>
-      <c r="C19" s="99"/>
+      <c r="C19" s="94"/>
       <c r="D19" s="66" t="s">
         <v>277</v>
       </c>
@@ -22825,7 +22819,7 @@
       <c r="E21" s="66" t="s">
         <v>343</v>
       </c>
-      <c r="I21" s="97"/>
+      <c r="I21" s="98"/>
       <c r="J21" s="67">
         <v>5</v>
       </c>
@@ -22837,7 +22831,7 @@
       </c>
     </row>
     <row r="22" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B22" s="101"/>
+      <c r="B22" s="97"/>
       <c r="C22" s="67">
         <v>3</v>
       </c>
@@ -22849,10 +22843,10 @@
       </c>
     </row>
     <row r="23" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="I23" s="93" t="s">
+      <c r="I23" s="99" t="s">
         <v>249</v>
       </c>
-      <c r="J23" s="94"/>
+      <c r="J23" s="100"/>
       <c r="K23" s="66" t="s">
         <v>277</v>
       </c>
@@ -22935,7 +22929,7 @@
       </c>
     </row>
     <row r="30" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="I30" s="97"/>
+      <c r="I30" s="98"/>
       <c r="J30" s="67">
         <v>7</v>
       </c>
@@ -22948,12 +22942,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B3:B17"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I17:I21"/>
     <mergeCell ref="I23:J23"/>
     <mergeCell ref="I24:I30"/>
     <mergeCell ref="N2:O2"/>
@@ -22962,6 +22950,12 @@
     <mergeCell ref="I3:I7"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="I10:I14"/>
+    <mergeCell ref="B3:B17"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I17:I21"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>